<commit_message>
Updating the model for Astro
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/IGCC_Netting_Flows.xlsx
+++ b/data_fetching/Entsoe/IGCC_Netting_Flows.xlsx
@@ -384,7 +384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -400,76 +400,76 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="B2">
-        <v>11.232</v>
+        <v>0.652</v>
       </c>
       <c r="C2">
-        <v>0.135</v>
+        <v>17.199</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2">
-        <v>46295.01041666666</v>
+        <v>46298.01041666666</v>
       </c>
       <c r="B3">
-        <v>2.381</v>
+        <v>0.163</v>
       </c>
       <c r="C3">
-        <v>5.156</v>
+        <v>2.254</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2">
-        <v>46295.02083333334</v>
+        <v>46298.02083333334</v>
       </c>
       <c r="B4">
-        <v>0.2</v>
+        <v>0.012</v>
       </c>
       <c r="C4">
-        <v>4.632</v>
+        <v>6.333</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2">
-        <v>46295.03125</v>
+        <v>46298.03125</v>
       </c>
       <c r="B5">
-        <v>0.059</v>
+        <v>0.194</v>
       </c>
       <c r="C5">
-        <v>2.1</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2">
-        <v>46295.04166666666</v>
+        <v>46298.04166666666</v>
       </c>
       <c r="B6">
-        <v>8.349</v>
+        <v>0.194</v>
       </c>
       <c r="C6">
-        <v>0.171</v>
+        <v>1.091</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2">
-        <v>46295.05208333334</v>
+        <v>46298.05208333334</v>
       </c>
       <c r="B7">
-        <v>5.505</v>
+        <v>6.123</v>
       </c>
       <c r="C7">
-        <v>3.063</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2">
-        <v>46295.0625</v>
+        <v>46298.0625</v>
       </c>
       <c r="B8">
-        <v>18.212</v>
+        <v>24.362</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -477,32 +477,32 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2">
-        <v>46295.07291666666</v>
+        <v>46298.07291666666</v>
       </c>
       <c r="B9">
-        <v>23.351</v>
+        <v>0.083</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>7.733</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2">
-        <v>46295.08333333334</v>
+        <v>46298.08333333334</v>
       </c>
       <c r="B10">
-        <v>5.773</v>
+        <v>1.988</v>
       </c>
       <c r="C10">
-        <v>0.028</v>
+        <v>0.478</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2">
-        <v>46295.09375</v>
+        <v>46298.09375</v>
       </c>
       <c r="B11">
-        <v>9.698</v>
+        <v>9.561999999999999</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -510,43 +510,43 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2">
-        <v>46295.10416666666</v>
+        <v>46298.10416666666</v>
       </c>
       <c r="B12">
-        <v>35.756</v>
+        <v>5.239</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="2">
-        <v>46295.11458333334</v>
+        <v>46298.11458333334</v>
       </c>
       <c r="B13">
-        <v>17.095</v>
+        <v>0.258</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>5.357</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="2">
-        <v>46295.125</v>
+        <v>46298.125</v>
       </c>
       <c r="B14">
-        <v>16.495</v>
+        <v>4.864</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="2">
-        <v>46295.13541666666</v>
+        <v>46298.13541666666</v>
       </c>
       <c r="B15">
-        <v>19.217</v>
+        <v>3.905</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -554,10 +554,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="2">
-        <v>46295.14583333334</v>
+        <v>46298.14583333334</v>
       </c>
       <c r="B16">
-        <v>24.425</v>
+        <v>6.35</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="2">
-        <v>46295.15625</v>
+        <v>46298.15625</v>
       </c>
       <c r="B17">
-        <v>37.883</v>
+        <v>10.297</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -576,10 +576,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="2">
-        <v>46295.16666666666</v>
+        <v>46298.16666666666</v>
       </c>
       <c r="B18">
-        <v>13.965</v>
+        <v>17.226</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -587,265 +587,210 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="2">
-        <v>46295.17708333334</v>
+        <v>46298.17708333334</v>
       </c>
       <c r="B19">
-        <v>9.773999999999999</v>
+        <v>1.975</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="2">
-        <v>46295.1875</v>
+        <v>46298.1875</v>
       </c>
       <c r="B20">
-        <v>3.764</v>
+        <v>3.482</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>1.343</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="2">
-        <v>46295.19791666666</v>
+        <v>46298.19791666666</v>
       </c>
       <c r="B21">
-        <v>4.44</v>
+        <v>27.439</v>
       </c>
       <c r="C21">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2">
-        <v>46295.20833333334</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>1.444</v>
       </c>
       <c r="C22">
-        <v>20.298</v>
+        <v>0.894</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2">
-        <v>46295.21875</v>
+        <v>46298.21875</v>
       </c>
       <c r="B23">
-        <v>1.534</v>
+        <v>5.032</v>
       </c>
       <c r="C23">
-        <v>16.983</v>
+        <v>0.288</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2">
-        <v>46295.22916666666</v>
+        <v>46298.22916666666</v>
       </c>
       <c r="B24">
-        <v>1.335</v>
+        <v>0.026</v>
       </c>
       <c r="C24">
-        <v>0.221</v>
+        <v>6.864</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2">
-        <v>46295.23958333334</v>
+        <v>46298.23958333334</v>
       </c>
       <c r="B25">
-        <v>5.091</v>
+        <v>0.197</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>7.578</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="2">
-        <v>46295.25</v>
+        <v>46298.25</v>
       </c>
       <c r="B26">
-        <v>0.651</v>
+        <v>1.562</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>0.641</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2">
-        <v>46295.26041666666</v>
+        <v>46298.26041666666</v>
       </c>
       <c r="B27">
-        <v>2.725</v>
+        <v>0.804</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>0.664</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2">
-        <v>46295.27083333334</v>
+        <v>46298.27083333334</v>
       </c>
       <c r="B28">
-        <v>30.741</v>
+        <v>0.252</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>0.212</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2">
-        <v>46295.28125</v>
+        <v>46298.28125</v>
       </c>
       <c r="B29">
-        <v>31.311</v>
+        <v>0.098</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>5.581</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="2">
-        <v>46295.29166666666</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="B30">
-        <v>8.467000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>6.278</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="2">
-        <v>46295.30208333334</v>
+        <v>46298.30208333334</v>
       </c>
       <c r="B31">
-        <v>11.85</v>
+        <v>0</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>13.374</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2">
-        <v>46295.3125</v>
+        <v>46298.3125</v>
       </c>
       <c r="B32">
-        <v>13.605</v>
+        <v>0</v>
       </c>
       <c r="C32">
-        <v>0</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="2">
-        <v>46295.32291666666</v>
+        <v>46298.32291666666</v>
       </c>
       <c r="B33">
-        <v>8.571999999999999</v>
+        <v>0</v>
       </c>
       <c r="C33">
-        <v>0.01</v>
+        <v>5.379</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="2">
-        <v>46295.33333333334</v>
+        <v>46298.33333333334</v>
       </c>
       <c r="B34">
-        <v>26.704</v>
+        <v>0.046</v>
       </c>
       <c r="C34">
-        <v>0.151</v>
+        <v>12.133</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="2">
-        <v>46295.34375</v>
+        <v>46298.34375</v>
       </c>
       <c r="B35">
-        <v>21.107</v>
+        <v>0</v>
       </c>
       <c r="C35">
-        <v>0.073</v>
+        <v>13.566</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2">
-        <v>46295.35416666666</v>
+        <v>46298.35416666666</v>
       </c>
       <c r="B36">
-        <v>4.749</v>
+        <v>2.73</v>
       </c>
       <c r="C36">
-        <v>0.237</v>
+        <v>8.824</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2">
-        <v>46295.36458333334</v>
+        <v>46298.36458333334</v>
       </c>
       <c r="B37">
-        <v>0.864</v>
+        <v>0</v>
       </c>
       <c r="C37">
-        <v>14.357</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="2">
-        <v>46295.375</v>
-      </c>
-      <c r="B38">
-        <v>7.365</v>
-      </c>
-      <c r="C38">
-        <v>0.044</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="2">
-        <v>46295.38541666666</v>
-      </c>
-      <c r="B39">
-        <v>0.323</v>
-      </c>
-      <c r="C39">
-        <v>8.962</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="2">
-        <v>46295.39583333334</v>
-      </c>
-      <c r="B40">
-        <v>0</v>
-      </c>
-      <c r="C40">
-        <v>8.558</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="2">
-        <v>46295.40625</v>
-      </c>
-      <c r="B41">
-        <v>0</v>
-      </c>
-      <c r="C41">
-        <v>50.093</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" s="2">
-        <v>46295.41666666666</v>
-      </c>
-      <c r="B42">
-        <v>0</v>
-      </c>
-      <c r="C42">
         <v>0</v>
       </c>
     </row>

</xml_diff>